<commit_message>
fix(1.1): MAD Override Flag — floor_override excludes intentional floors from instability detection (Montgomery 2019 Ch.6, Leys 2013)
</commit_message>
<xml_diff>
--- a/data/demo_tower_40floors.xlsx
+++ b/data/demo_tower_40floors.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,11 @@
           <t>panel_type</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>floor_override</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -487,6 +492,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -517,6 +525,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -547,6 +558,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -577,6 +591,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -607,6 +624,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -637,6 +657,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -667,6 +690,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -697,6 +723,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -727,6 +756,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -757,6 +789,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -787,6 +822,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -817,6 +855,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -847,6 +888,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -877,6 +921,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I15" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -907,6 +954,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I16" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -937,6 +987,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I17" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -967,6 +1020,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I18" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -997,6 +1053,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1027,6 +1086,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1057,6 +1119,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I21" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1087,6 +1152,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1117,6 +1185,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I23" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1147,6 +1218,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1177,6 +1251,9 @@
           <t>ALU-450</t>
         </is>
       </c>
+      <c r="I25" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1207,6 +1284,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1237,6 +1317,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I27" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1267,6 +1350,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I28" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1297,6 +1383,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1327,6 +1416,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I30" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1357,6 +1449,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I31" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1387,6 +1482,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1417,6 +1515,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I33" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1447,6 +1548,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I34" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1477,6 +1581,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I35" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1507,6 +1614,9 @@
           <t>H20-beam</t>
         </is>
       </c>
+      <c r="I36" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1537,6 +1647,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I37" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1567,6 +1680,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I38" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1597,6 +1713,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I39" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1627,6 +1746,9 @@
           <t>ALU-600</t>
         </is>
       </c>
+      <c r="I40" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1656,6 +1778,9 @@
         <is>
           <t>ALU-600</t>
         </is>
+      </c>
+      <c r="I41" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>